<commit_message>
📊 Update NAIC content history - 2026-03-03
</commit_message>
<xml_diff>
--- a/docs/content_history/pbr-2026-vm20-table-j-swaps.xlsx
+++ b/docs/content_history/pbr-2026-vm20-table-j-swaps.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29530"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\PBR\VM20_VM22_ProductSupport\PBR Production Web Data\Current Year\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0154C389-F2B5-45E1-AC30-CE3A57ABA9A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9676CA6-9403-4054-A6A3-9DD17EDDCE7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="795" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25180" windowHeight="16140" tabRatio="795" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="January_2026" sheetId="29" r:id="rId1"/>
-    <sheet name="LIBOR to SOFR Disclosure" sheetId="16" r:id="rId2"/>
-    <sheet name="LEGAL DISCLAIMER" sheetId="11" r:id="rId3"/>
+    <sheet name="February_2026" sheetId="30" r:id="rId1"/>
+    <sheet name="January_2026" sheetId="29" r:id="rId2"/>
+    <sheet name="LIBOR to SOFR Disclosure" sheetId="16" r:id="rId3"/>
+    <sheet name="LEGAL DISCLAIMER" sheetId="11" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -32,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="12">
   <si>
     <t>Weighted</t>
   </si>
@@ -65,6 +66,9 @@
   </si>
   <si>
     <t>** The  3 and 6 Month Current SOFR Swap Spreads are based on Term SOFR Rates obtained by contract from the CME Group.  The market data and all rights in and to it are the property of Chicago Mercantile Exchange Inc. or its licensors as applicable. All rights reserved, except as expressly licensed by Chicago Mercantile Exchange Inc.</t>
+  </si>
+  <si>
+    <t>Table J (02/27/2026) Swap Benchmark Spreads (in bps)</t>
   </si>
 </sst>
 </file>
@@ -147,7 +151,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" quotePrefix="1" applyFont="1" applyAlignment="1">
@@ -174,6 +178,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1617,21 +1622,432 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C73779D-48E1-4396-BCEC-CC77B9A96BB8}">
+  <dimension ref="A1:C39"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="3" width="19.6328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="6">
+        <v>6.6479016953999999</v>
+      </c>
+      <c r="C4" s="7">
+        <v>-8.4250997040000009</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="6">
+        <v>7.1046583332999997</v>
+      </c>
+      <c r="C5" s="6">
+        <v>-18.93440395</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="5">
+        <v>1</v>
+      </c>
+      <c r="B6" s="6">
+        <v>-2.926712974</v>
+      </c>
+      <c r="C6" s="6">
+        <v>-6.5887610170000004</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="5">
+        <v>2</v>
+      </c>
+      <c r="B7" s="6">
+        <v>-14.054845930000001</v>
+      </c>
+      <c r="C7" s="6">
+        <v>-9.7081414230000007</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="5">
+        <v>3</v>
+      </c>
+      <c r="B8" s="6">
+        <v>-19.05586533</v>
+      </c>
+      <c r="C8" s="6">
+        <v>-13.98810675</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" s="5">
+        <v>4</v>
+      </c>
+      <c r="B9" s="6">
+        <v>-21.562719229999999</v>
+      </c>
+      <c r="C9" s="6">
+        <v>-18.163567799999999</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" s="5">
+        <v>5</v>
+      </c>
+      <c r="B10" s="6">
+        <v>-24.50846623</v>
+      </c>
+      <c r="C10" s="6">
+        <v>-21.174162429999999</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" s="5">
+        <v>6</v>
+      </c>
+      <c r="B11" s="6">
+        <v>-29.26293536</v>
+      </c>
+      <c r="C11" s="6">
+        <v>-23.611543269999999</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" s="5">
+        <v>7</v>
+      </c>
+      <c r="B12" s="6">
+        <v>-33.452144599999997</v>
+      </c>
+      <c r="C12" s="6">
+        <v>-25.245948890000001</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" s="5">
+        <v>8</v>
+      </c>
+      <c r="B13" s="6">
+        <v>-36.257550690000002</v>
+      </c>
+      <c r="C13" s="6">
+        <v>-26.324832099999998</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A14" s="5">
+        <v>9</v>
+      </c>
+      <c r="B14" s="6">
+        <v>-38.687743159999997</v>
+      </c>
+      <c r="C14" s="6">
+        <v>-27.1029667</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A15" s="5">
+        <v>10</v>
+      </c>
+      <c r="B15" s="6">
+        <v>-40.57952607</v>
+      </c>
+      <c r="C15" s="6">
+        <v>-27.763705009999999</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A16" s="5">
+        <v>11</v>
+      </c>
+      <c r="B16" s="6">
+        <v>-43.304706379999999</v>
+      </c>
+      <c r="C16" s="6">
+        <v>-28.626325300000001</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A17" s="5">
+        <v>12</v>
+      </c>
+      <c r="B17" s="6">
+        <v>-47.412468269999998</v>
+      </c>
+      <c r="C17" s="6">
+        <v>-29.829543770000001</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A18" s="5">
+        <v>13</v>
+      </c>
+      <c r="B18" s="6">
+        <v>-51.459958409999999</v>
+      </c>
+      <c r="C18" s="6">
+        <v>-31.411004590000001</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A19" s="5">
+        <v>14</v>
+      </c>
+      <c r="B19" s="6">
+        <v>-54.779237950000002</v>
+      </c>
+      <c r="C19" s="6">
+        <v>-33.229500090000002</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A20" s="5">
+        <v>15</v>
+      </c>
+      <c r="B20" s="6">
+        <v>-57.657033689999999</v>
+      </c>
+      <c r="C20" s="6">
+        <v>-35.198334799999998</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A21" s="5">
+        <v>16</v>
+      </c>
+      <c r="B21" s="6">
+        <v>-60.051196099999999</v>
+      </c>
+      <c r="C21" s="6">
+        <v>-37.274791999999998</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A22" s="5">
+        <v>17</v>
+      </c>
+      <c r="B22" s="6">
+        <v>-61.971416550000001</v>
+      </c>
+      <c r="C22" s="6">
+        <v>-39.409508690000003</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A23" s="5">
+        <v>18</v>
+      </c>
+      <c r="B23" s="6">
+        <v>-63.46370709</v>
+      </c>
+      <c r="C23" s="6">
+        <v>-41.543833069999998</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A24" s="5">
+        <v>19</v>
+      </c>
+      <c r="B24" s="6">
+        <v>-64.639361570000005</v>
+      </c>
+      <c r="C24" s="6">
+        <v>-43.618617270000001</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A25" s="5">
+        <v>20</v>
+      </c>
+      <c r="B25" s="6">
+        <v>-65.546315149999998</v>
+      </c>
+      <c r="C25" s="6">
+        <v>-45.574980590000003</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A26" s="5">
+        <v>21</v>
+      </c>
+      <c r="B26" s="6">
+        <v>-66.269236430000007</v>
+      </c>
+      <c r="C26" s="6">
+        <v>-47.448015589999997</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A27" s="5">
+        <v>22</v>
+      </c>
+      <c r="B27" s="6">
+        <v>-66.873256389999995</v>
+      </c>
+      <c r="C27" s="6">
+        <v>-49.245376489999998</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A28" s="5">
+        <v>23</v>
+      </c>
+      <c r="B28" s="6">
+        <v>-67.405144989999997</v>
+      </c>
+      <c r="C28" s="6">
+        <v>-50.88986045</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A29" s="5">
+        <v>24</v>
+      </c>
+      <c r="B29" s="6">
+        <v>-67.899962639999998</v>
+      </c>
+      <c r="C29" s="6">
+        <v>-52.317818180000003</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A30" s="5">
+        <v>25</v>
+      </c>
+      <c r="B30" s="6">
+        <v>-68.393121019999995</v>
+      </c>
+      <c r="C30" s="6">
+        <v>-53.46845055</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A31" s="5">
+        <v>26</v>
+      </c>
+      <c r="B31" s="6">
+        <v>-68.919188009999999</v>
+      </c>
+      <c r="C31" s="6">
+        <v>-54.307336859999999</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A32" s="5">
+        <v>27</v>
+      </c>
+      <c r="B32" s="6">
+        <v>-69.427228479999997</v>
+      </c>
+      <c r="C32" s="6">
+        <v>-54.84603224</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A33" s="5">
+        <v>28</v>
+      </c>
+      <c r="B33" s="6">
+        <v>-69.967548239999999</v>
+      </c>
+      <c r="C33" s="6">
+        <v>-55.085355589999999</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A34" s="5">
+        <v>29</v>
+      </c>
+      <c r="B34" s="6">
+        <v>-70.560267899999999</v>
+      </c>
+      <c r="C34" s="6">
+        <v>-55.022050309999997</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A35" s="5">
+        <v>30</v>
+      </c>
+      <c r="B35" s="6">
+        <v>-71.285762520000006</v>
+      </c>
+      <c r="C35" s="6">
+        <v>-54.69621807</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A36" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B36" s="8">
+        <v>-46.996314603915621</v>
+      </c>
+      <c r="C36" s="8">
+        <v>-35.002318548249995</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A38" s="10"/>
+    </row>
+    <row r="39" spans="1:3" ht="66" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A39" s="10"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F39390C-8944-4BA3-A374-C71CF55A3914}">
   <dimension ref="A1:E39"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="3" width="19.7109375" customWidth="1"/>
+    <col min="1" max="3" width="19.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>8</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -1642,7 +2058,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="5" t="s">
         <v>3</v>
       </c>
@@ -1653,7 +2069,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
         <v>5</v>
       </c>
@@ -1664,7 +2080,7 @@
         <v>-8.4643284360000006</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="5" t="s">
         <v>6</v>
       </c>
@@ -1675,7 +2091,7 @@
         <v>-18.986706460000001</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="5">
         <v>1</v>
       </c>
@@ -1686,7 +2102,7 @@
         <v>-6.606153613</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="5">
         <v>2</v>
       </c>
@@ -1697,7 +2113,7 @@
         <v>-9.6725825039999993</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="5">
         <v>3</v>
       </c>
@@ -1708,7 +2124,7 @@
         <v>-13.90377076</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="5">
         <v>4</v>
       </c>
@@ -1719,7 +2135,7 @@
         <v>-18.05126491</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="5">
         <v>5</v>
       </c>
@@ -1730,7 +2146,7 @@
         <v>-21.058171550000001</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" s="5">
         <v>6</v>
       </c>
@@ -1741,7 +2157,7 @@
         <v>-23.482340529999998</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" s="5">
         <v>7</v>
       </c>
@@ -1752,7 +2168,7 @@
         <v>-25.112373340000001</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" s="5">
         <v>8</v>
       </c>
@@ -1763,7 +2179,7 @@
         <v>-26.207170059999999</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" s="5">
         <v>9</v>
       </c>
@@ -1774,7 +2190,7 @@
         <v>-27.01171896</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" s="5">
         <v>10</v>
       </c>
@@ -1785,7 +2201,7 @@
         <v>-27.699147780000001</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" s="5">
         <v>11</v>
       </c>
@@ -1796,7 +2212,7 @@
         <v>-28.582440519999999</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" s="5">
         <v>12</v>
       </c>
@@ -1807,7 +2223,7 @@
         <v>-29.797805400000001</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" s="5">
         <v>13</v>
       </c>
@@ -1818,7 +2234,7 @@
         <v>-31.38552271</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" s="5">
         <v>14</v>
       </c>
@@ -1829,7 +2245,7 @@
         <v>-33.206359569999996</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" s="5">
         <v>15</v>
       </c>
@@ -1840,7 +2256,7 @@
         <v>-35.175185190000001</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" s="5">
         <v>16</v>
       </c>
@@ -1851,7 +2267,7 @@
         <v>-37.250174440000002</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" s="5">
         <v>17</v>
       </c>
@@ -1862,7 +2278,7 @@
         <v>-39.383293340000002</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A23" s="5">
         <v>18</v>
       </c>
@@ -1873,7 +2289,7 @@
         <v>-41.514898170000002</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A24" s="5">
         <v>19</v>
       </c>
@@ -1884,7 +2300,7 @@
         <v>-43.58589877</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25" s="5">
         <v>20</v>
       </c>
@@ -1895,7 +2311,7 @@
         <v>-45.536655600000003</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A26" s="5">
         <v>21</v>
       </c>
@@ -1906,7 +2322,7 @@
         <v>-47.402761550000001</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A27" s="5">
         <v>22</v>
       </c>
@@ -1917,7 +2333,7 @@
         <v>-49.193163900000002</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A28" s="5">
         <v>23</v>
       </c>
@@ -1928,7 +2344,7 @@
         <v>-50.831508980000002</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A29" s="5">
         <v>24</v>
       </c>
@@ -1939,7 +2355,7 @@
         <v>-52.254304140000002</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A30" s="5">
         <v>25</v>
       </c>
@@ -1950,7 +2366,7 @@
         <v>-53.401048920000001</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A31" s="5">
         <v>26</v>
       </c>
@@ -1961,7 +2377,7 @@
         <v>-54.237701129999998</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A32" s="5">
         <v>27</v>
       </c>
@@ -1972,7 +2388,7 @@
         <v>-54.776711149999997</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" s="5">
         <v>28</v>
       </c>
@@ -1983,7 +2399,7 @@
         <v>-55.018984750000001</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" s="5">
         <v>29</v>
       </c>
@@ -1994,7 +2410,7 @@
         <v>-54.961556510000001</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" s="5">
         <v>30</v>
       </c>
@@ -2005,7 +2421,7 @@
         <v>-54.64476792</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" s="5" t="s">
         <v>7</v>
       </c>
@@ -2016,12 +2432,12 @@
         <v>-34.949889736343749</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="39" spans="1:5" ht="66" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" ht="66" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="9" t="s">
         <v>10</v>
       </c>
@@ -2038,28 +2454,28 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F25262A5-84B2-4BF6-AF4E-DBAA1AC8379B}">
   <sheetPr codeName="Sheet8">
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr codeName="Sheet7">
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
   <dimension ref="H31"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="31" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="31" spans="8:8" x14ac:dyDescent="0.35">
       <c r="H31" s="1"/>
     </row>
   </sheetData>

</xml_diff>